<commit_message>
[ADD] First optimization of MLP
</commit_message>
<xml_diff>
--- a/results/metrics_modelling4_6-neural_networks.xlsx
+++ b/results/metrics_modelling4_6-neural_networks.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DH5"/>
+  <dimension ref="A1:DH7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2548,6 +2548,786 @@
       </c>
       <c r="DH5" t="n">
         <v>0.009537194934686195</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CategoryEmbeddingModel_splashing_smote_opt-model</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>{'estimator': 'PytorchTabularEstimator', 'estimator_params': {'model_class': 'CategoryEmbeddingModelConfig', 'trainer_config_params': {'max_epochs': 300, 'batch_size': 300, 'early_stopping': 'valid_loss', 'early_stopping_patience': 10, 'accelerator': 'gpu', 'devices': 1, 'progress_bar': 'none'}, 'optimizer_config_params': {'optimizer': 'Adam', 'lr_scheduler': 'ReduceLROnPlateau', 'lr_scheduler_params': {'patience': 5, 'factor': 0.5}}, 'model_config_params': {'activation': 'LeakyReLU', 'dropout': 0.05368731404192041, 'learning_rate': 0.010100246162580432, 'use_batch_norm': False, 'batch_norm_continuous_input': True, 'layers': '128'}}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.8775510204081632</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.8865979381443299</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.9220679012345679</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.8395253841665045</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.8368055555555556</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.8076923076923077</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.7924528301886792</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.8922558922558923</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.8854166666666666</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.9139784946236558</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.9593005952380952</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.8849171752397558</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.8950892857142857</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.811965811965812</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.9047619047619048</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.8558558558558558</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>1.0455152988433838, 2.822162389755249, 0.9511258602142334, 1.748558521270752, 1.6606271266937256, 1.165550947189331, 1.687471866607666</t>
+        </is>
+      </c>
+      <c r="Z6" t="n">
+        <v>1.583001715796334</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>1.660627126693726</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0.5906765900268036</v>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>0.021254301071166992, 0.03110504150390625, 0.03519082069396973, 0.03544902801513672, 0.031102895736694336, 0.03302192687988281, 0.030825138092041016</t>
+        </is>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.03113559314182826</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0.03110504150390625</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0.004413407554968602</v>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>0.9444444444444444, 0.7735849056603774, 0.9056603773584906, 0.8490566037735849, 0.9622641509433962, 0.8490566037735849, 0.8301886792452831</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>0.9330827067669173, 0.7611111111111111, 0.903250773993808, 0.8475232198142415, 0.9473684210526316, 0.8591331269349844, 0.8212074303405572</t>
+        </is>
+      </c>
+      <c r="AI6" t="n">
+        <v>0.8675252557163216</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0.8591331269349844</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0.06081452303130598</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>0.873465109314166</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>0.8490566037735849</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>0.06210627511558647</v>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>0.9577464788732395, 0.823529411764706, 0.9253731343283583, 0.8787878787878787, 0.9714285714285714, 0.8749999999999999, 0.8656716417910447</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>0.918918918918919, 0.6842105263157895, 0.8717948717948718, 0.8, 0.9444444444444444, 0.8095238095238095, 0.7692307692307692</t>
+        </is>
+      </c>
+      <c r="AQ6" t="n">
+        <v>0.8283033343183719</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>0.8095238095238095</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>0.0836638768397777</v>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>0.9383326988960792, 0.7538699690402477, 0.898584003061615, 0.8393939393939394, 0.9579365079365079, 0.8422619047619047, 0.8174512055109069</t>
+        </is>
+      </c>
+      <c r="AU6" t="n">
+        <v>0.8639757469430286</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>0.8422619047619047</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>0.06646038969565106</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>0.8996481595676855</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>0.8787878787878787</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>0.04954185412513377</v>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>0.9444444444444444, 0.8484848484848485, 0.9393939393939394, 0.90625, 0.9444444444444444, 0.9333333333333333, 0.8787878787878788</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>0.9444444444444444, 0.65, 0.85, 0.7619047619047619, 1.0, 0.7391304347826086, 0.75</t>
+        </is>
+      </c>
+      <c r="BC6" t="n">
+        <v>0.8136399487331164</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>0.7619047619047619</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>0.1147781781500156</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>0.9135912698412698</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>0.03477145784916613</v>
+      </c>
+      <c r="BI6" t="inlineStr">
+        <is>
+          <t>0.9714285714285714, 0.8, 0.9117647058823529, 0.8529411764705882, 1.0, 0.8235294117647058, 0.8529411764705882</t>
+        </is>
+      </c>
+      <c r="BJ6" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.7222222222222222, 0.8947368421052632, 0.8421052631578947, 0.8947368421052632, 0.8947368421052632, 0.7894736842105263</t>
+        </is>
+      </c>
+      <c r="BK6" t="n">
+        <v>0.8475355054302423</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>0.06326356014833588</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>0.8875150060024009</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>0.8529411764705882</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>0.07012859637223683</v>
+      </c>
+      <c r="BQ6" t="inlineStr">
+        <is>
+          <t>0.9834586466165414, 0.8777777777777778, 0.9860681114551083, 0.9226006191950464, 0.9628482972136223, 0.9071207430340558, 0.8978328173374615</t>
+        </is>
+      </c>
+      <c r="BR6" t="n">
+        <v>0.9339581446613734</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>0.9226006191950464</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>0.04019755084189896</v>
+      </c>
+      <c r="BU6" t="inlineStr">
+        <is>
+          <t>0.8584905660377359, 0.9341692789968652, 0.8652037617554859, 0.9028213166144201, 0.8996865203761756, 0.8840125391849529, 0.9059561128526645</t>
+        </is>
+      </c>
+      <c r="BV6" t="inlineStr">
+        <is>
+          <t>0.872372113101662, 0.9312580231065468, 0.8736575307156972, 0.9047813386029728, 0.8923661826617407, 0.8862230432167713, 0.9132013059541197</t>
+        </is>
+      </c>
+      <c r="BW6" t="n">
+        <v>0.8962656481942159</v>
+      </c>
+      <c r="BX6" t="n">
+        <v>0.8923661826617407</v>
+      </c>
+      <c r="BY6" t="n">
+        <v>0.01993520765672447</v>
+      </c>
+      <c r="BZ6" t="n">
+        <v>0.8929057279740429</v>
+      </c>
+      <c r="CA6" t="n">
+        <v>0.8996865203761756</v>
+      </c>
+      <c r="CB6" t="n">
+        <v>0.02404811350633178</v>
+      </c>
+      <c r="CC6" t="inlineStr">
+        <is>
+          <t>0.8825065274151435, 0.9484029484029484, 0.8900255754475703, 0.9226932668329177, 0.921951219512195, 0.9072681704260651, 0.9242424242424243</t>
+        </is>
+      </c>
+      <c r="CD6" t="inlineStr">
+        <is>
+          <t>0.8221343873517787, 0.9090909090909091, 0.8259109311740891, 0.8691983122362869, 0.8596491228070176, 0.8451882845188284, 0.8760330578512397</t>
+        </is>
+      </c>
+      <c r="CE6" t="n">
+        <v>0.8581721435757357</v>
+      </c>
+      <c r="CF6" t="n">
+        <v>0.8596491228070176</v>
+      </c>
+      <c r="CG6" t="n">
+        <v>0.0281414211708796</v>
+      </c>
+      <c r="CH6" t="inlineStr">
+        <is>
+          <t>0.8523204573834611, 0.9287469287469288, 0.8579682533108297, 0.8959457895346024, 0.8908001711596063, 0.8762282274724468, 0.9001377410468321</t>
+        </is>
+      </c>
+      <c r="CI6" t="n">
+        <v>0.8860210812363867</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>0.8908001711596063</v>
+      </c>
+      <c r="CK6" t="n">
+        <v>0.0243917751141534</v>
+      </c>
+      <c r="CL6" t="n">
+        <v>0.9138700188970379</v>
+      </c>
+      <c r="CM6" t="n">
+        <v>0.9219512195121951</v>
+      </c>
+      <c r="CN6" t="n">
+        <v>0.0208363556074919</v>
+      </c>
+      <c r="CO6" t="inlineStr">
+        <is>
+          <t>0.949438202247191, 0.9554455445544554, 0.9405405405405406, 0.9487179487179487, 0.9264705882352942, 0.9378238341968912, 0.9631578947368421</t>
+        </is>
+      </c>
+      <c r="CP6" t="inlineStr">
+        <is>
+          <t>0.7428571428571429, 0.8974358974358975, 0.7611940298507462, 0.8306451612903226, 0.8521739130434782, 0.8015873015873016, 0.8217054263565892</t>
+        </is>
+      </c>
+      <c r="CQ6" t="n">
+        <v>0.8153712674887824</v>
+      </c>
+      <c r="CR6" t="n">
+        <v>0.8217054263565892</v>
+      </c>
+      <c r="CS6" t="n">
+        <v>0.04891088204035585</v>
+      </c>
+      <c r="CT6" t="n">
+        <v>0.9459420790327375</v>
+      </c>
+      <c r="CU6" t="n">
+        <v>0.9487179487179487</v>
+      </c>
+      <c r="CV6" t="n">
+        <v>0.01121765170544328</v>
+      </c>
+      <c r="CW6" t="inlineStr">
+        <is>
+          <t>0.824390243902439, 0.9414634146341463, 0.8446601941747572, 0.8980582524271845, 0.9174757281553398, 0.8786407766990292, 0.8883495145631068</t>
+        </is>
+      </c>
+      <c r="CX6" t="inlineStr">
+        <is>
+          <t>0.9203539823008849, 0.9210526315789473, 0.9026548672566371, 0.911504424778761, 0.8672566371681416, 0.8938053097345132, 0.9380530973451328</t>
+        </is>
+      </c>
+      <c r="CY6" t="n">
+        <v>0.9078115643090026</v>
+      </c>
+      <c r="CZ6" t="n">
+        <v>0.911504424778761</v>
+      </c>
+      <c r="DA6" t="n">
+        <v>0.02113999073337604</v>
+      </c>
+      <c r="DB6" t="n">
+        <v>0.884719732079429</v>
+      </c>
+      <c r="DC6" t="n">
+        <v>0.8883495145631068</v>
+      </c>
+      <c r="DD6" t="n">
+        <v>0.03735019536015502</v>
+      </c>
+      <c r="DE6" t="inlineStr">
+        <is>
+          <t>0.9502482192963523, 0.9822849807445443, 0.9425423146318412, 0.972656585617321, 0.9707663888650228, 0.9600481140991494, 0.9749763725405962</t>
+        </is>
+      </c>
+      <c r="DF6" t="n">
+        <v>0.9647889965421182</v>
+      </c>
+      <c r="DG6" t="n">
+        <v>0.9707663888650228</v>
+      </c>
+      <c r="DH6" t="n">
+        <v>0.01328987420691922</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CategoryEmbeddingModel_no_fragmentation_smotenc_opt-model</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>{'estimator': 'PytorchTabularEstimator', 'estimator_params': {'model_class': 'CategoryEmbeddingModelConfig', 'trainer_config_params': {'max_epochs': 300, 'batch_size': 300, 'early_stopping': 'valid_loss', 'early_stopping_patience': 10, 'accelerator': 'gpu', 'devices': 1, 'progress_bar': 'none'}, 'optimizer_config_params': {'optimizer': 'Adam', 'lr_scheduler': 'ReduceLROnPlateau', 'lr_scheduler_params': {'patience': 5, 'factor': 0.5}}, 'model_config_params': {'activation': 'LeakyReLU', 'dropout': 0.020012990188122446, 'learning_rate': 0.051818480542551844, 'use_batch_norm': False, 'batch_norm_continuous_input': True, 'layers': '128'}}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.8933333333333333</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.7894736842105262</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.9572727272727273</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.8590225563909774</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.8477272727272727</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.9122807017543859</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.9454545454545454</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.9285714285714285</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.9393939393939394</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.8674698795180723</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.9113924050632911</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0.9806642666356985</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.9236111111111112</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0.9304668447334804</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.9672897196261683</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0.9495412844036697</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>1.2609286308288574, 1.5858442783355713, 1.6516401767730713, 0.9509181976318359, 1.1848039627075195, 1.284769058227539, 1.8354003429412842</t>
+        </is>
+      </c>
+      <c r="Z7" t="n">
+        <v>1.39347209249224</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>1.284769058227539</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0.2847903623229752</v>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>0.09030795097351074, 0.03214716911315918, 0.03312182426452637, 0.0426630973815918, 0.03192734718322754, 0.016433000564575195, 0.03195929527282715</t>
+        </is>
+      </c>
+      <c r="AD7" t="n">
+        <v>0.03979424067905971</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0.03214716911315918</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0.02181705110790425</v>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>0.9074074074074074, 0.8867924528301887, 0.9622641509433962, 0.9245283018867925, 0.8867924528301887, 0.8867924528301887, 0.9433962264150944</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>0.9153846153846155, 0.9001831501831502, 0.9514652014652014, 0.9258241758241759, 0.8315018315018314, 0.8315018315018314, 0.9615384615384616</t>
+        </is>
+      </c>
+      <c r="AI7" t="n">
+        <v>0.9024856096284667</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>0.9153846153846155</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0.04881452885379466</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>0.9139962064490368</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>0.9074074074074074</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>0.02820492758291179</v>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>0.8484848484848485, 0.8125000000000001, 0.9285714285714286, 0.8666666666666666, 0.7692307692307692, 0.7692307692307692, 0.9032258064516129</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>0.9333333333333333, 0.9189189189189189, 0.9743589743589743, 0.9473684210526315, 0.9249999999999999, 0.9249999999999999, 0.9600000000000001</t>
+        </is>
+      </c>
+      <c r="AQ7" t="n">
+        <v>0.9405685210948368</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0.01916628981964416</v>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>0.8909090909090909, 0.8657094594594594, 0.9514652014652014, 0.9070175438596491, 0.8471153846153845, 0.8471153846153845, 0.9316129032258065</t>
+        </is>
+      </c>
+      <c r="AU7" t="n">
+        <v>0.891563566878568</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>0.8909090909090909</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>0.03789294241633237</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>0.8425586126622994</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>0.8484848484848485</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>0.05775873079532773</v>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>0.7777777777777778, 0.7222222222222222, 0.9285714285714286, 0.8125, 0.8333333333333334, 0.8333333333333334, 0.8235294117647058</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>0.9722222222222222, 0.9714285714285714, 0.9743589743589743, 0.972972972972973, 0.9024390243902439, 0.9024390243902439, 1.0</t>
+        </is>
+      </c>
+      <c r="BC7" t="n">
+        <v>0.956551541394747</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>0.9722222222222222</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>0.03545170133409956</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>0.8187525010004001</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>0.8235294117647058</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>0.05799548443661851</v>
+      </c>
+      <c r="BI7" t="inlineStr">
+        <is>
+          <t>0.9333333333333333, 0.9285714285714286, 0.9285714285714286, 0.9285714285714286, 0.7142857142857143, 0.7142857142857143, 1.0</t>
+        </is>
+      </c>
+      <c r="BJ7" t="inlineStr">
+        <is>
+          <t>0.8974358974358975, 0.8717948717948718, 0.9743589743589743, 0.9230769230769231, 0.9487179487179487, 0.9487179487179487, 0.9230769230769231</t>
+        </is>
+      </c>
+      <c r="BK7" t="n">
+        <v>0.9267399267399269</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>0.03193332559370455</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>0.8782312925170068</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>0.9285714285714286</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>0.106383770352787</v>
+      </c>
+      <c r="BQ7" t="inlineStr">
+        <is>
+          <t>0.9692307692307692, 0.9322344322344323, 0.9835164835164836, 0.9487179487179487, 0.9725274725274725, 0.9413919413919414, 0.9926739926739927</t>
+        </is>
+      </c>
+      <c r="BR7" t="n">
+        <v>0.9628990057561486</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>0.9692307692307692</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>0.0208682982459598</v>
+      </c>
+      <c r="BU7" t="inlineStr">
+        <is>
+          <t>0.9150943396226415, 0.9529780564263323, 0.9310344827586207, 0.9122257053291536, 0.9310344827586207, 0.9310344827586207, 0.9278996865203761</t>
+        </is>
+      </c>
+      <c r="BV7" t="inlineStr">
+        <is>
+          <t>0.9270451770451771, 0.9604575163398692, 0.9380090497737557, 0.8952237305178481, 0.9267722473604827, 0.9492458521870286, 0.9321266968325792</t>
+        </is>
+      </c>
+      <c r="BW7" t="n">
+        <v>0.9326971814366772</v>
+      </c>
+      <c r="BX7" t="n">
+        <v>0.9321266968325792</v>
+      </c>
+      <c r="BY7" t="n">
+        <v>0.01906509756698112</v>
+      </c>
+      <c r="BZ7" t="n">
+        <v>0.9287573194534807</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>0.9310344827586207</v>
+      </c>
+      <c r="CB7" t="n">
+        <v>0.01232249589354134</v>
+      </c>
+      <c r="CC7" t="inlineStr">
+        <is>
+          <t>0.8556149732620322, 0.9171270718232044, 0.8804347826086957, 0.8390804597701149, 0.8764044943820225, 0.8842105263157894, 0.8743169398907105</t>
+        </is>
+      </c>
+      <c r="CD7" t="inlineStr">
+        <is>
+          <t>0.9398663697104677, 0.9671772428884027, 0.9515418502202644, 0.939655172413793, 0.9521739130434783, 0.9508928571428572, 0.9494505494505495</t>
+        </is>
+      </c>
+      <c r="CE7" t="n">
+        <v>0.9501082792671163</v>
+      </c>
+      <c r="CF7" t="n">
+        <v>0.9508928571428572</v>
+      </c>
+      <c r="CG7" t="n">
+        <v>0.008559738087521994</v>
+      </c>
+      <c r="CH7" t="inlineStr">
+        <is>
+          <t>0.8977406714862499, 0.9421521573558036, 0.91598831641448, 0.889367816091954, 0.9142892037127504, 0.9175516917293234, 0.91188374467063</t>
+        </is>
+      </c>
+      <c r="CI7" t="n">
+        <v>0.9127105144944557</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>0.9142892037127504</v>
+      </c>
+      <c r="CK7" t="n">
+        <v>0.01546029427372632</v>
+      </c>
+      <c r="CL7" t="n">
+        <v>0.8753127497217957</v>
+      </c>
+      <c r="CM7" t="n">
+        <v>0.8764044943820225</v>
+      </c>
+      <c r="CN7" t="n">
+        <v>0.02254141571874112</v>
+      </c>
+      <c r="CO7" t="inlineStr">
+        <is>
+          <t>0.7766990291262136, 0.8645833333333334, 0.8181818181818182, 0.8202247191011236, 0.8387096774193549, 0.8, 0.8163265306122449</t>
+        </is>
+      </c>
+      <c r="CP7" t="inlineStr">
+        <is>
+          <t>0.9813953488372092, 0.9910313901345291, 0.9818181818181818, 0.9478260869565217, 0.9690265486725663, 0.9953271028037384, 0.9773755656108597</t>
+        </is>
+      </c>
+      <c r="CQ7" t="n">
+        <v>0.977685746404801</v>
+      </c>
+      <c r="CR7" t="n">
+        <v>0.9813953488372092</v>
+      </c>
+      <c r="CS7" t="n">
+        <v>0.01457414057581606</v>
+      </c>
+      <c r="CT7" t="n">
+        <v>0.8192464439677269</v>
+      </c>
+      <c r="CU7" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="CV7" t="n">
+        <v>0.02570596221319831</v>
+      </c>
+      <c r="CW7" t="inlineStr">
+        <is>
+          <t>0.9523809523809523, 0.9764705882352941, 0.9529411764705882, 0.8588235294117647, 0.9176470588235294, 0.9882352941176471, 0.9411764705882353</t>
+        </is>
+      </c>
+      <c r="CX7" t="inlineStr">
+        <is>
+          <t>0.9017094017094017, 0.9444444444444444, 0.9230769230769231, 0.9316239316239316, 0.9358974358974359, 0.9102564102564102, 0.9230769230769231</t>
+        </is>
+      </c>
+      <c r="CY7" t="n">
+        <v>0.9242979242979245</v>
+      </c>
+      <c r="CZ7" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="DA7" t="n">
+        <v>0.01365120865384486</v>
+      </c>
+      <c r="DB7" t="n">
+        <v>0.9410964385754301</v>
+      </c>
+      <c r="DC7" t="n">
+        <v>0.9523809523809523</v>
+      </c>
+      <c r="DD7" t="n">
+        <v>0.03974876751322907</v>
+      </c>
+      <c r="DE7" t="inlineStr">
+        <is>
+          <t>0.9783272283272283, 0.9855203619909502, 0.9809954751131222, 0.9697838109602814, 0.9786324786324787, 0.9828557063851181, 0.9814982403217698</t>
+        </is>
+      </c>
+      <c r="DF7" t="n">
+        <v>0.9796590431044213</v>
+      </c>
+      <c r="DG7" t="n">
+        <v>0.9809954751131222</v>
+      </c>
+      <c r="DH7" t="n">
+        <v>0.004630491909295781</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[ADD] MLP optimization with 1000 iterations
</commit_message>
<xml_diff>
--- a/results/metrics_modelling4_6-neural_networks.xlsx
+++ b/results/metrics_modelling4_6-neural_networks.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DH7"/>
+  <dimension ref="A1:DH6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2568,766 +2568,376 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>{'estimator': 'PytorchTabularEstimator', 'estimator_params': {'model_class': 'CategoryEmbeddingModelConfig', 'trainer_config_params': {'max_epochs': 300, 'batch_size': 300, 'early_stopping': 'valid_loss', 'early_stopping_patience': 10, 'accelerator': 'gpu', 'devices': 1, 'progress_bar': 'none'}, 'optimizer_config_params': {'optimizer': 'Adam', 'lr_scheduler': 'ReduceLROnPlateau', 'lr_scheduler_params': {'patience': 5, 'factor': 0.5}}, 'model_config_params': {'activation': 'LeakyReLU', 'dropout': 0.05368731404192041, 'learning_rate': 0.010100246162580432, 'use_batch_norm': False, 'batch_norm_continuous_input': True, 'layers': '128'}}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
+          <t>{'estimator': 'PytorchTabularEstimator', 'estimator_params': {'model_class': 'CategoryEmbeddingModelConfig', 'trainer_config_params': {'max_epochs': 300, 'batch_size': 300, 'early_stopping': 'valid_loss', 'early_stopping_patience': 10, 'accelerator': 'gpu', 'devices': 1, 'progress_bar': 'none'}, 'optimizer_config_params': {'optimizer': 'Adam', 'lr_scheduler': 'ReduceLROnPlateau', 'lr_scheduler_params': {'patience': 5, 'factor': 0.5}}, 'model_config_params': {'activation': 'ReLU', 'dropout': 0.12063675406353806, 'learning_rate': 0.010999581868953563, 'use_batch_norm': False, 'batch_norm_continuous_input': True, 'layers': '128'}}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {}, 'random_state': 42}</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.8533333333333334</v>
+        <v>0.8133333333333334</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8775510204081632</v>
+        <v>0.8269230769230769</v>
       </c>
       <c r="G6" t="n">
         <v>0.8958333333333334</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8865979381443299</v>
+        <v>0.86</v>
       </c>
       <c r="I6" t="n">
-        <v>0.9220679012345679</v>
+        <v>0.8958333333333334</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8395253841665045</v>
+        <v>0.79</v>
       </c>
       <c r="K6" t="n">
-        <v>0.8368055555555556</v>
+        <v>0.78125</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8076923076923077</v>
+        <v>0.7826086956521739</v>
       </c>
       <c r="M6" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="N6" t="n">
-        <v>0.7924528301886792</v>
+        <v>0.72</v>
       </c>
       <c r="O6" t="n">
-        <v>0.8922558922558923</v>
+        <v>0.9023569023569024</v>
       </c>
       <c r="P6" t="n">
-        <v>0.9444444444444444</v>
+        <v>0.9267015706806283</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.8854166666666666</v>
+        <v>0.921875</v>
       </c>
       <c r="R6" t="n">
-        <v>0.9139784946236558</v>
+        <v>0.9242819843342037</v>
       </c>
       <c r="S6" t="n">
-        <v>0.9593005952380952</v>
+        <v>0.952951388888889</v>
       </c>
       <c r="T6" t="n">
-        <v>0.8849171752397558</v>
+        <v>0.8934206130201825</v>
       </c>
       <c r="U6" t="n">
-        <v>0.8950892857142857</v>
+        <v>0.8942708333333333</v>
       </c>
       <c r="V6" t="n">
-        <v>0.811965811965812</v>
+        <v>0.8584905660377359</v>
       </c>
       <c r="W6" t="n">
-        <v>0.9047619047619048</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="X6" t="n">
-        <v>0.8558558558558558</v>
+        <v>0.8625592417061612</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>1.0455152988433838, 2.822162389755249, 0.9511258602142334, 1.748558521270752, 1.6606271266937256, 1.165550947189331, 1.687471866607666</t>
+          <t>1.2052509784698486, 1.2054443359375, 1.2191855907440186, 1.5888311862945557, 2.6861276626586914, 1.4826538562774658, 1.9853689670562744</t>
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>1.583001715796334</v>
+        <v>1.624694653919765</v>
       </c>
       <c r="AA6" t="n">
-        <v>1.660627126693726</v>
+        <v>1.482653856277466</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.5906765900268036</v>
+        <v>0.5062931385532728</v>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>0.021254301071166992, 0.03110504150390625, 0.03519082069396973, 0.03544902801513672, 0.031102895736694336, 0.03302192687988281, 0.030825138092041016</t>
+          <t>0.0312504768371582, 0.03312563896179199, 0.031681060791015625, 0.030777692794799805, 0.0356142520904541, 0.03489208221435547, 0.033148765563964844</t>
         </is>
       </c>
       <c r="AD6" t="n">
-        <v>0.03113559314182826</v>
+        <v>0.03292713846479144</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.03110504150390625</v>
+        <v>0.03312563896179199</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.004413407554968602</v>
+        <v>0.001696808982661119</v>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>0.9444444444444444, 0.7735849056603774, 0.9056603773584906, 0.8490566037735849, 0.9622641509433962, 0.8490566037735849, 0.8301886792452831</t>
+          <t>0.9444444444444444, 0.8113207547169812, 0.9056603773584906, 0.8679245283018868, 0.9245283018867925, 0.8113207547169812, 0.8113207547169812</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>0.9330827067669173, 0.7611111111111111, 0.903250773993808, 0.8475232198142415, 0.9473684210526316, 0.8591331269349844, 0.8212074303405572</t>
+          <t>0.9330827067669173, 0.8031746031746032, 0.914860681114551, 0.8738390092879257, 0.9179566563467492, 0.8297213622291022, 0.794891640866873</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>0.8675252557163216</v>
+        <v>0.8667895228266745</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.8591331269349844</v>
+        <v>0.8738390092879257</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.06081452303130598</v>
+        <v>0.0534035917342563</v>
       </c>
       <c r="AL6" t="n">
-        <v>0.873465109314166</v>
+        <v>0.868074273734651</v>
       </c>
       <c r="AM6" t="n">
-        <v>0.8490566037735849</v>
+        <v>0.8679245283018868</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.06210627511558647</v>
+        <v>0.05357915858245822</v>
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>0.9577464788732395, 0.823529411764706, 0.9253731343283583, 0.8787878787878787, 0.9714285714285714, 0.8749999999999999, 0.8656716417910447</t>
+          <t>0.9577464788732395, 0.8529411764705883, 0.923076923076923, 0.8923076923076922, 0.9411764705882353, 0.8387096774193549, 0.8529411764705882</t>
         </is>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>0.918918918918919, 0.6842105263157895, 0.8717948717948718, 0.8, 0.9444444444444444, 0.8095238095238095, 0.7692307692307692</t>
+          <t>0.918918918918919, 0.7368421052631577, 0.8780487804878049, 0.8292682926829269, 0.8947368421052632, 0.7727272727272727, 0.7368421052631579</t>
         </is>
       </c>
       <c r="AQ6" t="n">
-        <v>0.8283033343183719</v>
+        <v>0.8239120453497859</v>
       </c>
       <c r="AR6" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.8292682926829269</v>
       </c>
       <c r="AS6" t="n">
-        <v>0.0836638768397777</v>
+        <v>0.07049231287323876</v>
       </c>
       <c r="AT6" t="inlineStr">
         <is>
-          <t>0.9383326988960792, 0.7538699690402477, 0.898584003061615, 0.8393939393939394, 0.9579365079365079, 0.8422619047619047, 0.8174512055109069</t>
+          <t>0.9383326988960792, 0.794891640866873, 0.900562851782364, 0.8607879924953096, 0.9179566563467492, 0.8057184750733137, 0.794891640866873</t>
         </is>
       </c>
       <c r="AU6" t="n">
-        <v>0.8639757469430286</v>
+        <v>0.859020279475366</v>
       </c>
       <c r="AV6" t="n">
-        <v>0.8422619047619047</v>
+        <v>0.8607879924953096</v>
       </c>
       <c r="AW6" t="n">
-        <v>0.06646038969565106</v>
+        <v>0.05676884639655286</v>
       </c>
       <c r="AX6" t="n">
-        <v>0.8996481595676855</v>
+        <v>0.8941285136009459</v>
       </c>
       <c r="AY6" t="n">
-        <v>0.8787878787878787</v>
+        <v>0.8923076923076922</v>
       </c>
       <c r="AZ6" t="n">
-        <v>0.04954185412513377</v>
+        <v>0.04402292008056208</v>
       </c>
       <c r="BA6" t="inlineStr">
         <is>
-          <t>0.9444444444444444, 0.8484848484848485, 0.9393939393939394, 0.90625, 0.9444444444444444, 0.9333333333333333, 0.8787878787878788</t>
+          <t>0.9444444444444444, 0.8787878787878788, 0.967741935483871, 0.9354838709677419, 0.9411764705882353, 0.9285714285714286, 0.8529411764705882</t>
         </is>
       </c>
       <c r="BB6" t="inlineStr">
         <is>
-          <t>0.9444444444444444, 0.65, 0.85, 0.7619047619047619, 1.0, 0.7391304347826086, 0.75</t>
+          <t>0.9444444444444444, 0.7, 0.8181818181818182, 0.7727272727272727, 0.8947368421052632, 0.68, 0.7368421052631579</t>
         </is>
       </c>
       <c r="BC6" t="n">
-        <v>0.8136399487331164</v>
+        <v>0.7924189261031366</v>
       </c>
       <c r="BD6" t="n">
-        <v>0.7619047619047619</v>
+        <v>0.7727272727272727</v>
       </c>
       <c r="BE6" t="n">
-        <v>0.1147781781500156</v>
+        <v>0.09172961653360312</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.9135912698412698</v>
+        <v>0.9213067436163126</v>
       </c>
       <c r="BG6" t="n">
-        <v>0.9333333333333333</v>
+        <v>0.9354838709677419</v>
       </c>
       <c r="BH6" t="n">
-        <v>0.03477145784916613</v>
+        <v>0.03745827682372321</v>
       </c>
       <c r="BI6" t="inlineStr">
         <is>
-          <t>0.9714285714285714, 0.8, 0.9117647058823529, 0.8529411764705882, 1.0, 0.8235294117647058, 0.8529411764705882</t>
+          <t>0.9714285714285714, 0.8285714285714286, 0.8823529411764706, 0.8529411764705882, 0.9411764705882353, 0.7647058823529411, 0.8529411764705882</t>
         </is>
       </c>
       <c r="BJ6" t="inlineStr">
         <is>
-          <t>0.8947368421052632, 0.7222222222222222, 0.8947368421052632, 0.8421052631578947, 0.8947368421052632, 0.8947368421052632, 0.7894736842105263</t>
+          <t>0.8947368421052632, 0.7777777777777778, 0.9473684210526315, 0.8947368421052632, 0.8947368421052632, 0.8947368421052632, 0.7368421052631579</t>
         </is>
       </c>
       <c r="BK6" t="n">
-        <v>0.8475355054302423</v>
+        <v>0.8629908103592313</v>
       </c>
       <c r="BL6" t="n">
         <v>0.8947368421052632</v>
       </c>
       <c r="BM6" t="n">
-        <v>0.06326356014833588</v>
+        <v>0.07002609720867461</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.8875150060024009</v>
+        <v>0.8705882352941176</v>
       </c>
       <c r="BO6" t="n">
         <v>0.8529411764705882</v>
       </c>
       <c r="BP6" t="n">
-        <v>0.07012859637223683</v>
+        <v>0.06424195640580728</v>
       </c>
       <c r="BQ6" t="inlineStr">
         <is>
-          <t>0.9834586466165414, 0.8777777777777778, 0.9860681114551083, 0.9226006191950464, 0.9628482972136223, 0.9071207430340558, 0.8978328173374615</t>
+          <t>0.9849624060150375, 0.8634920634920634, 0.9860681114551083, 0.931888544891641, 0.958204334365325, 0.9040247678018576, 0.890092879256966</t>
         </is>
       </c>
       <c r="BR6" t="n">
-        <v>0.9339581446613734</v>
+        <v>0.9312475867539998</v>
       </c>
       <c r="BS6" t="n">
-        <v>0.9226006191950464</v>
+        <v>0.931888544891641</v>
       </c>
       <c r="BT6" t="n">
-        <v>0.04019755084189896</v>
+        <v>0.04414788711856033</v>
       </c>
       <c r="BU6" t="inlineStr">
         <is>
-          <t>0.8584905660377359, 0.9341692789968652, 0.8652037617554859, 0.9028213166144201, 0.8996865203761756, 0.8840125391849529, 0.9059561128526645</t>
+          <t>0.8584905660377359, 0.890282131661442, 0.8589341692789969, 0.9059561128526645, 0.9153605015673981, 0.8746081504702194, 0.9122257053291536</t>
         </is>
       </c>
       <c r="BV6" t="inlineStr">
         <is>
-          <t>0.872372113101662, 0.9312580231065468, 0.8736575307156972, 0.9047813386029728, 0.8923661826617407, 0.8862230432167713, 0.9132013059541197</t>
+          <t>0.872372113101662, 0.889323919554985, 0.8688031617836584, 0.9092061173640347, 0.9104948878769654, 0.8769438955236704, 0.9140604862960735</t>
         </is>
       </c>
       <c r="BW6" t="n">
-        <v>0.8962656481942159</v>
+        <v>0.8916006545001498</v>
       </c>
       <c r="BX6" t="n">
-        <v>0.8923661826617407</v>
+        <v>0.889323919554985</v>
       </c>
       <c r="BY6" t="n">
-        <v>0.01993520765672447</v>
+        <v>0.01805093984900737</v>
       </c>
       <c r="BZ6" t="n">
-        <v>0.8929057279740429</v>
+        <v>0.8879796195996587</v>
       </c>
       <c r="CA6" t="n">
-        <v>0.8996865203761756</v>
+        <v>0.890282131661442</v>
       </c>
       <c r="CB6" t="n">
-        <v>0.02404811350633178</v>
+        <v>0.02254544582770811</v>
       </c>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>0.8825065274151435, 0.9484029484029484, 0.8900255754475703, 0.9226932668329177, 0.921951219512195, 0.9072681704260651, 0.9242424242424243</t>
+          <t>0.8825065274151435, 0.9127182044887782, 0.884318766066838, 0.9250000000000002, 0.9339853300733497, 0.8994974874371858, 0.9303482587064676</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>0.8221343873517787, 0.9090909090909091, 0.8259109311740891, 0.8691983122362869, 0.8596491228070176, 0.8451882845188284, 0.8760330578512397</t>
+          <t>0.8221343873517787, 0.8523206751054853, 0.8192771084337348, 0.8739495798319328, 0.8820960698689956, 0.8333333333333335, 0.8813559322033898</t>
         </is>
       </c>
       <c r="CE6" t="n">
-        <v>0.8581721435757357</v>
+        <v>0.8520667265898073</v>
       </c>
       <c r="CF6" t="n">
-        <v>0.8596491228070176</v>
+        <v>0.8523206751054853</v>
       </c>
       <c r="CG6" t="n">
-        <v>0.0281414211708796</v>
+        <v>0.02552474091963724</v>
       </c>
       <c r="CH6" t="inlineStr">
         <is>
-          <t>0.8523204573834611, 0.9287469287469288, 0.8579682533108297, 0.8959457895346024, 0.8908001711596063, 0.8762282274724468, 0.9001377410468321</t>
+          <t>0.8523204573834611, 0.8825194397971317, 0.8517979372502864, 0.8994747899159665, 0.9080406999711726, 0.8664154103852597, 0.9058520954549287</t>
         </is>
       </c>
       <c r="CI6" t="n">
-        <v>0.8860210812363867</v>
+        <v>0.8809172614511723</v>
       </c>
       <c r="CJ6" t="n">
-        <v>0.8908001711596063</v>
+        <v>0.8825194397971317</v>
       </c>
       <c r="CK6" t="n">
-        <v>0.0243917751141534</v>
+        <v>0.02261602349554817</v>
       </c>
       <c r="CL6" t="n">
-        <v>0.9138700188970379</v>
+        <v>0.9097677963125375</v>
       </c>
       <c r="CM6" t="n">
-        <v>0.9219512195121951</v>
+        <v>0.9127182044887782</v>
       </c>
       <c r="CN6" t="n">
-        <v>0.0208363556074919</v>
+        <v>0.01981009294751581</v>
       </c>
       <c r="CO6" t="inlineStr">
         <is>
-          <t>0.949438202247191, 0.9554455445544554, 0.9405405405405406, 0.9487179487179487, 0.9264705882352942, 0.9378238341968912, 0.9631578947368421</t>
+          <t>0.949438202247191, 0.9336734693877551, 0.9398907103825137, 0.9536082474226805, 0.9408866995073891, 0.9322916666666666, 0.9540816326530612</t>
         </is>
       </c>
       <c r="CP6" t="inlineStr">
         <is>
-          <t>0.7428571428571429, 0.8974358974358975, 0.7611940298507462, 0.8306451612903226, 0.8521739130434782, 0.8015873015873016, 0.8217054263565892</t>
+          <t>0.7428571428571429, 0.8211382113821138, 0.75, 0.832, 0.8706896551724138, 0.7874015748031497, 0.8455284552845529</t>
         </is>
       </c>
       <c r="CQ6" t="n">
-        <v>0.8153712674887824</v>
+        <v>0.8070878627856247</v>
       </c>
       <c r="CR6" t="n">
-        <v>0.8217054263565892</v>
+        <v>0.8211382113821138</v>
       </c>
       <c r="CS6" t="n">
-        <v>0.04891088204035585</v>
+        <v>0.04490156442906437</v>
       </c>
       <c r="CT6" t="n">
-        <v>0.9459420790327375</v>
+        <v>0.9434100897524653</v>
       </c>
       <c r="CU6" t="n">
-        <v>0.9487179487179487</v>
+        <v>0.9408866995073891</v>
       </c>
       <c r="CV6" t="n">
-        <v>0.01121765170544328</v>
+        <v>0.008378518668209902</v>
       </c>
       <c r="CW6" t="inlineStr">
         <is>
-          <t>0.824390243902439, 0.9414634146341463, 0.8446601941747572, 0.8980582524271845, 0.9174757281553398, 0.8786407766990292, 0.8883495145631068</t>
+          <t>0.824390243902439, 0.8926829268292683, 0.8349514563106796, 0.8980582524271845, 0.9271844660194175, 0.8689320388349514, 0.9077669902912622</t>
         </is>
       </c>
       <c r="CX6" t="inlineStr">
         <is>
-          <t>0.9203539823008849, 0.9210526315789473, 0.9026548672566371, 0.911504424778761, 0.8672566371681416, 0.8938053097345132, 0.9380530973451328</t>
+          <t>0.9203539823008849, 0.8859649122807017, 0.9026548672566371, 0.9203539823008849, 0.8938053097345132, 0.8849557522123894, 0.9203539823008849</t>
         </is>
       </c>
       <c r="CY6" t="n">
-        <v>0.9078115643090026</v>
+        <v>0.9040632554838423</v>
       </c>
       <c r="CZ6" t="n">
-        <v>0.911504424778761</v>
+        <v>0.9026548672566371</v>
       </c>
       <c r="DA6" t="n">
-        <v>0.02113999073337604</v>
+        <v>0.01509975901910118</v>
       </c>
       <c r="DB6" t="n">
-        <v>0.884719732079429</v>
+        <v>0.8791380535164574</v>
       </c>
       <c r="DC6" t="n">
-        <v>0.8883495145631068</v>
+        <v>0.8926829268292683</v>
       </c>
       <c r="DD6" t="n">
-        <v>0.03735019536015502</v>
+        <v>0.03530166337841305</v>
       </c>
       <c r="DE6" t="inlineStr">
         <is>
-          <t>0.9502482192963523, 0.9822849807445443, 0.9425423146318412, 0.972656585617321, 0.9707663888650228, 0.9600481140991494, 0.9749763725405962</t>
+          <t>0.9486941506583207, 0.9559264013692769, 0.9454205687773864, 0.963119683821634, 0.9765228971561131, 0.9630122862788899, 0.9745467823696194</t>
         </is>
       </c>
       <c r="DF6" t="n">
-        <v>0.9647889965421182</v>
+        <v>0.9610346814901772</v>
       </c>
       <c r="DG6" t="n">
-        <v>0.9707663888650228</v>
+        <v>0.9630122862788899</v>
       </c>
       <c r="DH6" t="n">
-        <v>0.01328987420691922</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>df_dimless</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>no_fragmentation</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CategoryEmbeddingModel_no_fragmentation_smotenc_opt-model</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>{'estimator': 'PytorchTabularEstimator', 'estimator_params': {'model_class': 'CategoryEmbeddingModelConfig', 'trainer_config_params': {'max_epochs': 300, 'batch_size': 300, 'early_stopping': 'valid_loss', 'early_stopping_patience': 10, 'accelerator': 'gpu', 'devices': 1, 'progress_bar': 'none'}, 'optimizer_config_params': {'optimizer': 'Adam', 'lr_scheduler': 'ReduceLROnPlateau', 'lr_scheduler_params': {'patience': 5, 'factor': 0.5}}, 'model_config_params': {'activation': 'LeakyReLU', 'dropout': 0.020012990188122446, 'learning_rate': 0.051818480542551844, 'use_batch_norm': False, 'batch_norm_continuous_input': True, 'layers': '128'}}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': True, 'smote_params': {'categorical_features': ('wettability', 'inclination')}, 'random_state': 42}</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>0.8933333333333333</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.7894736842105262</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.9572727272727273</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.8590225563909774</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.8477272727272727</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.9122807017543859</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0.9454545454545454</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.9285714285714285</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0.9393939393939394</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0.8674698795180723</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0.9113924050632911</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.9806642666356985</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0.9236111111111112</v>
-      </c>
-      <c r="U7" t="n">
-        <v>0.9304668447334804</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0.9672897196261683</v>
-      </c>
-      <c r="W7" t="n">
-        <v>0.9495412844036697</v>
-      </c>
-      <c r="X7" t="n">
-        <v>0.9583333333333334</v>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>1.2609286308288574, 1.5858442783355713, 1.6516401767730713, 0.9509181976318359, 1.1848039627075195, 1.284769058227539, 1.8354003429412842</t>
-        </is>
-      </c>
-      <c r="Z7" t="n">
-        <v>1.39347209249224</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>1.284769058227539</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>0.2847903623229752</v>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>0.09030795097351074, 0.03214716911315918, 0.03312182426452637, 0.0426630973815918, 0.03192734718322754, 0.016433000564575195, 0.03195929527282715</t>
-        </is>
-      </c>
-      <c r="AD7" t="n">
-        <v>0.03979424067905971</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>0.03214716911315918</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>0.02181705110790425</v>
-      </c>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>0.9074074074074074, 0.8867924528301887, 0.9622641509433962, 0.9245283018867925, 0.8867924528301887, 0.8867924528301887, 0.9433962264150944</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>0.9153846153846155, 0.9001831501831502, 0.9514652014652014, 0.9258241758241759, 0.8315018315018314, 0.8315018315018314, 0.9615384615384616</t>
-        </is>
-      </c>
-      <c r="AI7" t="n">
-        <v>0.9024856096284667</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>0.9153846153846155</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>0.04881452885379466</v>
-      </c>
-      <c r="AL7" t="n">
-        <v>0.9139962064490368</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>0.9074074074074074</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>0.02820492758291179</v>
-      </c>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>0.8484848484848485, 0.8125000000000001, 0.9285714285714286, 0.8666666666666666, 0.7692307692307692, 0.7692307692307692, 0.9032258064516129</t>
-        </is>
-      </c>
-      <c r="AP7" t="inlineStr">
-        <is>
-          <t>0.9333333333333333, 0.9189189189189189, 0.9743589743589743, 0.9473684210526315, 0.9249999999999999, 0.9249999999999999, 0.9600000000000001</t>
-        </is>
-      </c>
-      <c r="AQ7" t="n">
-        <v>0.9405685210948368</v>
-      </c>
-      <c r="AR7" t="n">
-        <v>0.9333333333333333</v>
-      </c>
-      <c r="AS7" t="n">
-        <v>0.01916628981964416</v>
-      </c>
-      <c r="AT7" t="inlineStr">
-        <is>
-          <t>0.8909090909090909, 0.8657094594594594, 0.9514652014652014, 0.9070175438596491, 0.8471153846153845, 0.8471153846153845, 0.9316129032258065</t>
-        </is>
-      </c>
-      <c r="AU7" t="n">
-        <v>0.891563566878568</v>
-      </c>
-      <c r="AV7" t="n">
-        <v>0.8909090909090909</v>
-      </c>
-      <c r="AW7" t="n">
-        <v>0.03789294241633237</v>
-      </c>
-      <c r="AX7" t="n">
-        <v>0.8425586126622994</v>
-      </c>
-      <c r="AY7" t="n">
-        <v>0.8484848484848485</v>
-      </c>
-      <c r="AZ7" t="n">
-        <v>0.05775873079532773</v>
-      </c>
-      <c r="BA7" t="inlineStr">
-        <is>
-          <t>0.7777777777777778, 0.7222222222222222, 0.9285714285714286, 0.8125, 0.8333333333333334, 0.8333333333333334, 0.8235294117647058</t>
-        </is>
-      </c>
-      <c r="BB7" t="inlineStr">
-        <is>
-          <t>0.9722222222222222, 0.9714285714285714, 0.9743589743589743, 0.972972972972973, 0.9024390243902439, 0.9024390243902439, 1.0</t>
-        </is>
-      </c>
-      <c r="BC7" t="n">
-        <v>0.956551541394747</v>
-      </c>
-      <c r="BD7" t="n">
-        <v>0.9722222222222222</v>
-      </c>
-      <c r="BE7" t="n">
-        <v>0.03545170133409956</v>
-      </c>
-      <c r="BF7" t="n">
-        <v>0.8187525010004001</v>
-      </c>
-      <c r="BG7" t="n">
-        <v>0.8235294117647058</v>
-      </c>
-      <c r="BH7" t="n">
-        <v>0.05799548443661851</v>
-      </c>
-      <c r="BI7" t="inlineStr">
-        <is>
-          <t>0.9333333333333333, 0.9285714285714286, 0.9285714285714286, 0.9285714285714286, 0.7142857142857143, 0.7142857142857143, 1.0</t>
-        </is>
-      </c>
-      <c r="BJ7" t="inlineStr">
-        <is>
-          <t>0.8974358974358975, 0.8717948717948718, 0.9743589743589743, 0.9230769230769231, 0.9487179487179487, 0.9487179487179487, 0.9230769230769231</t>
-        </is>
-      </c>
-      <c r="BK7" t="n">
-        <v>0.9267399267399269</v>
-      </c>
-      <c r="BL7" t="n">
-        <v>0.9230769230769231</v>
-      </c>
-      <c r="BM7" t="n">
-        <v>0.03193332559370455</v>
-      </c>
-      <c r="BN7" t="n">
-        <v>0.8782312925170068</v>
-      </c>
-      <c r="BO7" t="n">
-        <v>0.9285714285714286</v>
-      </c>
-      <c r="BP7" t="n">
-        <v>0.106383770352787</v>
-      </c>
-      <c r="BQ7" t="inlineStr">
-        <is>
-          <t>0.9692307692307692, 0.9322344322344323, 0.9835164835164836, 0.9487179487179487, 0.9725274725274725, 0.9413919413919414, 0.9926739926739927</t>
-        </is>
-      </c>
-      <c r="BR7" t="n">
-        <v>0.9628990057561486</v>
-      </c>
-      <c r="BS7" t="n">
-        <v>0.9692307692307692</v>
-      </c>
-      <c r="BT7" t="n">
-        <v>0.0208682982459598</v>
-      </c>
-      <c r="BU7" t="inlineStr">
-        <is>
-          <t>0.9150943396226415, 0.9529780564263323, 0.9310344827586207, 0.9122257053291536, 0.9310344827586207, 0.9310344827586207, 0.9278996865203761</t>
-        </is>
-      </c>
-      <c r="BV7" t="inlineStr">
-        <is>
-          <t>0.9270451770451771, 0.9604575163398692, 0.9380090497737557, 0.8952237305178481, 0.9267722473604827, 0.9492458521870286, 0.9321266968325792</t>
-        </is>
-      </c>
-      <c r="BW7" t="n">
-        <v>0.9326971814366772</v>
-      </c>
-      <c r="BX7" t="n">
-        <v>0.9321266968325792</v>
-      </c>
-      <c r="BY7" t="n">
-        <v>0.01906509756698112</v>
-      </c>
-      <c r="BZ7" t="n">
-        <v>0.9287573194534807</v>
-      </c>
-      <c r="CA7" t="n">
-        <v>0.9310344827586207</v>
-      </c>
-      <c r="CB7" t="n">
-        <v>0.01232249589354134</v>
-      </c>
-      <c r="CC7" t="inlineStr">
-        <is>
-          <t>0.8556149732620322, 0.9171270718232044, 0.8804347826086957, 0.8390804597701149, 0.8764044943820225, 0.8842105263157894, 0.8743169398907105</t>
-        </is>
-      </c>
-      <c r="CD7" t="inlineStr">
-        <is>
-          <t>0.9398663697104677, 0.9671772428884027, 0.9515418502202644, 0.939655172413793, 0.9521739130434783, 0.9508928571428572, 0.9494505494505495</t>
-        </is>
-      </c>
-      <c r="CE7" t="n">
-        <v>0.9501082792671163</v>
-      </c>
-      <c r="CF7" t="n">
-        <v>0.9508928571428572</v>
-      </c>
-      <c r="CG7" t="n">
-        <v>0.008559738087521994</v>
-      </c>
-      <c r="CH7" t="inlineStr">
-        <is>
-          <t>0.8977406714862499, 0.9421521573558036, 0.91598831641448, 0.889367816091954, 0.9142892037127504, 0.9175516917293234, 0.91188374467063</t>
-        </is>
-      </c>
-      <c r="CI7" t="n">
-        <v>0.9127105144944557</v>
-      </c>
-      <c r="CJ7" t="n">
-        <v>0.9142892037127504</v>
-      </c>
-      <c r="CK7" t="n">
-        <v>0.01546029427372632</v>
-      </c>
-      <c r="CL7" t="n">
-        <v>0.8753127497217957</v>
-      </c>
-      <c r="CM7" t="n">
-        <v>0.8764044943820225</v>
-      </c>
-      <c r="CN7" t="n">
-        <v>0.02254141571874112</v>
-      </c>
-      <c r="CO7" t="inlineStr">
-        <is>
-          <t>0.7766990291262136, 0.8645833333333334, 0.8181818181818182, 0.8202247191011236, 0.8387096774193549, 0.8, 0.8163265306122449</t>
-        </is>
-      </c>
-      <c r="CP7" t="inlineStr">
-        <is>
-          <t>0.9813953488372092, 0.9910313901345291, 0.9818181818181818, 0.9478260869565217, 0.9690265486725663, 0.9953271028037384, 0.9773755656108597</t>
-        </is>
-      </c>
-      <c r="CQ7" t="n">
-        <v>0.977685746404801</v>
-      </c>
-      <c r="CR7" t="n">
-        <v>0.9813953488372092</v>
-      </c>
-      <c r="CS7" t="n">
-        <v>0.01457414057581606</v>
-      </c>
-      <c r="CT7" t="n">
-        <v>0.8192464439677269</v>
-      </c>
-      <c r="CU7" t="n">
-        <v>0.8181818181818182</v>
-      </c>
-      <c r="CV7" t="n">
-        <v>0.02570596221319831</v>
-      </c>
-      <c r="CW7" t="inlineStr">
-        <is>
-          <t>0.9523809523809523, 0.9764705882352941, 0.9529411764705882, 0.8588235294117647, 0.9176470588235294, 0.9882352941176471, 0.9411764705882353</t>
-        </is>
-      </c>
-      <c r="CX7" t="inlineStr">
-        <is>
-          <t>0.9017094017094017, 0.9444444444444444, 0.9230769230769231, 0.9316239316239316, 0.9358974358974359, 0.9102564102564102, 0.9230769230769231</t>
-        </is>
-      </c>
-      <c r="CY7" t="n">
-        <v>0.9242979242979245</v>
-      </c>
-      <c r="CZ7" t="n">
-        <v>0.9230769230769231</v>
-      </c>
-      <c r="DA7" t="n">
-        <v>0.01365120865384486</v>
-      </c>
-      <c r="DB7" t="n">
-        <v>0.9410964385754301</v>
-      </c>
-      <c r="DC7" t="n">
-        <v>0.9523809523809523</v>
-      </c>
-      <c r="DD7" t="n">
-        <v>0.03974876751322907</v>
-      </c>
-      <c r="DE7" t="inlineStr">
-        <is>
-          <t>0.9783272283272283, 0.9855203619909502, 0.9809954751131222, 0.9697838109602814, 0.9786324786324787, 0.9828557063851181, 0.9814982403217698</t>
-        </is>
-      </c>
-      <c r="DF7" t="n">
-        <v>0.9796590431044213</v>
-      </c>
-      <c r="DG7" t="n">
-        <v>0.9809954751131222</v>
-      </c>
-      <c r="DH7" t="n">
-        <v>0.004630491909295781</v>
+        <v>0.01103826845198495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>